<commit_message>
Réunit le contexte et la proposition IA dans la feuille de relecture humaine
</commit_message>
<xml_diff>
--- a/annotation/exemples_ia_20.xlsx
+++ b/annotation/exemples_ia_20.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Commentaires" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Positions IA" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exemples fictifs" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relecture humaine" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Guide" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Commentaires" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Positions IA" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Exemples fictifs" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Relecture humaine" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Guide'!$A$1:$B$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Commentaires'!$A$1:$O$101</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Positions IA'!$A$1:$K$101</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Exemples fictifs'!$A$1:$G$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Relecture humaine'!$A$1:$G$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Relecture humaine'!$A$1:$J$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -47,7 +47,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -57,6 +57,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00244766"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1F5FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF5CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -73,7 +83,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -82,6 +92,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -448,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -548,6 +567,18 @@
       <c r="B8" t="inlineStr">
         <is>
           <t>Textes non tronqués pour préserver le sens; peuvent contenir des données personnelles et des propos offensants.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Lecture simplifiée</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Ouvrir Relecture humaine : commentaire, parent et proposition IA sont réunis sur chaque ligne. Colonnes bleutées : lecture; colonnes jaunes : vos annotations. Un commentaire à plusieurs positions est répété. Les textes complets sont conservés; agrandir la barre de formule si un texte dépasse la hauteur maximale Excel.</t>
         </is>
       </c>
     </row>
@@ -3953,343 +3984,858 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
-    <col width="75" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="56" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="45" customWidth="1" min="9" max="9"/>
+    <col width="50" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>position_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>commentaire_complet</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>commentaire_parent</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>proposition_IA_et_justification</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>accord</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>correction_acteur</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>correction_objet</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>correction_position</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>correction_preuve</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>note</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="2" ht="168" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>C001-P1</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr"/>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Les gaz il était puissant</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Aucun parent : commentaire principal.</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Acteur : police
+Objet : usage de la force
+Position : décrit sans position
+Preuve : Les gaz il était puissant
+Incertitude : contexte insuffisant
+Note IA : Constate la puissance des gaz; ne dit pas explicitement si leur usage est légitime.</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="n"/>
+      <c r="F2" s="6" t="n"/>
+      <c r="G2" s="6" t="n"/>
+      <c r="H2" s="6" t="n"/>
+      <c r="I2" s="6" t="n"/>
+      <c r="J2" s="6" t="n"/>
+    </row>
+    <row r="3" ht="224" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>C002-P1</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr"/>
-      <c r="C3" s="2" t="inlineStr"/>
-      <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>@wizzfred2 relancé des pavés deja lancer par des flics manifestnts! sachant en plus qu'un manifestant qui lance un pavé sur un flic c'est légal, un policier qui lance un pavé sur un manifestant c'est illégale!</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>pardon mais le blouson pour ce protéger des pavés c'est pour quoi? genre un pavé ca fait mal 🤣 genre y a des manifestants qui lancent des pavés🤣</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Acteur : police
+Objet : usage de la force
+Position : condamne
+Preuve : un policier qui lance un pavé sur un manifestant c'est illégale!
+Incertitude : lecture explicite
+Responsabilité attribuée : Policiers décrits comme lançant des pavés
+Argument : Opposition de légalité entre gestes des policiers et manifestants
+Note IA : Argument juridique de l’auteur, non vérifié; contexte du parent utile.</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="n"/>
+      <c r="F3" s="6" t="n"/>
+      <c r="G3" s="6" t="n"/>
+      <c r="H3" s="6" t="n"/>
+      <c r="I3" s="6" t="n"/>
+      <c r="J3" s="6" t="n"/>
+    </row>
+    <row r="4" ht="196" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>C002-P2</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr"/>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>@wizzfred2 relancé des pavés deja lancer par des flics manifestnts! sachant en plus qu'un manifestant qui lance un pavé sur un flic c'est légal, un policier qui lance un pavé sur un manifestant c'est illégale!</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>pardon mais le blouson pour ce protéger des pavés c'est pour quoi? genre un pavé ca fait mal 🤣 genre y a des manifestants qui lancent des pavés🤣</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Acteur : manifestants
+Objet : violences et dégâts
+Position : justifie ou soutient
+Preuve : un manifestant qui lance un pavé sur un flic c'est légal
+Incertitude : lecture explicite
+Argument : Légalité alléguée du jet de pavé sur un policier
+Note IA : Propos de l’auteur, pas une conclusion juridique du rapport.</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="6" t="n"/>
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="n"/>
+      <c r="I4" s="6" t="n"/>
+      <c r="J4" s="6" t="n"/>
+    </row>
+    <row r="5" ht="409" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>C003-P1</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr"/>
-      <c r="C5" s="2" t="inlineStr"/>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>PFFFF,LA génération Z,ils ont bien trouvé leurs surnoms:Z,Comme Zéros, Zouaves,vraiment, vous n'êtes pas gèners,rien ne vous déranges dans vos actes nombrilistes,qui a casser vos écoles???,qui brosses les cours???,qui fous la merde???,Vous etes des touts petits microbes qui ne savez que vous plaindres,oui,des punaises de lits,voilà ce que vous êtes...des🧟‍♂️🧟‍♀️🧟 ZOMBIES,qui ne savez que suivre sans réfléchir part vous mêmes parce qu'il est plus gait de (manifester),tout casser avec les casseurs qui ont foutus vos écoles en l'air,et qui font pareils avec les commerces et les biens d'autruits,vous dansez,vous criez,vous revendiquez mais dans les actes,que faites vous de concrets?Vous voulez touts sans l'avoir gagner...Foutez nous la paix et foutez vous en l'air si ça vous chantes,mais,cessez d'etres aussi cons!!! Pitié pour ceux qui ont travaillers commes des bêtes pour que vous soyez biens,pour que vous n'ayez pas a travailler plustot que d'aller a l'école vous instruires!!! Vous vivez toujours chez papa/maman,assister et vous trouvez que c'est pas assez,vous voulez le beurre et l'argent du beurre sans rien faire,SI...sortir,vous starers la gueules avec touts ce qui passes,vous ozez dires que vous etes malheureux a causes de vos ainés...plaignez vous...vous ne vous levez pas a 4heure du matin pour aller travailler pour manger?,ou parce que votre boulot est a 100km de chez vous et qu'il faut être a l'heure et user le1/3 de votre salaire a payer les transports car pas de fric pour une voiture...Non,vraiment, vous n'êtes pas a plaindres...et les droits que vous avez(mais c'est jamais assez),c'est grâce aux manifestations de vos parents et grands parents qui eux,n'ont pas piliers les commerces pour ce faires entendre...Oui,la France va mal,on c'est tous fait avoir part Minimacron et sa pédo,mais plutôt que d'etres plus intelligents,vous mettez de l'eau aux moulins que vous dites combattres!!! La vie,c'est pas les réseaux sociaux, c'est tout autour de vous...ouvrez les yeux!!!et c'est pas parce que vous n'êtes pas de droites que vous etes de gauche et vis et versa...GÉNÉRATON ZÉROS ‼️‼️‼️ARRÊTEZ D'ÉCOUTER VOS(STARS)et pensez part vous mêmes,vous avez le droit de ne pas êtres en accords avec touts ceux qui restent derrière leurs écrans alors que vous,vous êtes dans la rue,parce que c'est ce qu'il va arriver...vous en doutez???On peux encore sauver la France avant qu'elle ne devienne un Brésil n°2,un pays de NON DROITS, vous savez ce que c'est⁉️Allez voire sur vos st réseaux...si c'est vraiment ça que vous voulez,et provoquez par votre ignorance...Et puis merde,débrouillez vous la gen Z...😮‍💨😮‍💨😮‍💨🤐😶🤫🫡😾💋💟</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Aucun parent : commentaire principal.</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Acteur : manifestants
+Objet : violences et dégâts
+Position : condamne
+Preuve : tout casser avec les casseurs qui ont foutus vos écoles en l'air
+Incertitude : lecture explicite
+Responsabilité attribuée : Jeunes participants associés aux casseurs et dégradations
+Argument : Dégradations des écoles, commerces et biens
+Note IA : Texte hostile aux jeunes manifestants; aucune position sur la force policière déduite.</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="6" t="n"/>
+      <c r="I5" s="6" t="n"/>
+      <c r="J5" s="6" t="n"/>
+    </row>
+    <row r="6" ht="196" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>C004-P1</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr"/>
-      <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>😭😭😭😭😭😭 a quoi peuvent servir les centaures sur des émeutes aussi violentes avec des groupes de casseurs très mobiles? Réponse ils ne servent a que dalle sur ce type d émeute....plutôt des boulets car s ils sont encerclés et pris a partie par les émeutiers, il faudra les protéger....</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Ils sont oû les CENTAURES blindés de la gendarmerie !!! 💥💥</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Acteur : police
+Objet : protection et sécurité
+Position : condamne
+Preuve : ils ne servent a que dalle sur ce type d émeute
+Incertitude : lecture explicite
+Argument : Véhicules blindés jugés inutiles et vulnérables face à des groupes mobiles
+Note IA : Critique de l’efficacité du matériel, pas une condamnation générale de la police. Titre évoquant le 18 octobre.</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
+      <c r="I6" s="6" t="n"/>
+      <c r="J6" s="6" t="n"/>
+    </row>
+    <row r="7" ht="224" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>C005-P1</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr"/>
-      <c r="C7" s="2" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>FACT: When humans needs are not met due to “ no livable wages “ that ensure at least a comfortable life, THEN violence, rage and distain for capitalists will continue to rise!</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Aucun parent : commentaire principal.</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Acteur : autre
+Objet : violences et dégâts
+Position : décrit sans position
+Preuve : THEN violence, rage and distain for capitalists will continue to rise!
+Incertitude : ambigu
+Responsabilité attribuée : Conditions salariales insuffisantes présentées comme cause de violences
+Argument : Besoins humains non satisfaits et salaires insuffisants
+Note IA : Explication causale; ne suffit pas à conclure à une approbation des violences. Commentaire anglais; pas spécifiquement policier.</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="6" t="n"/>
+      <c r="I7" s="6" t="n"/>
+      <c r="J7" s="6" t="n"/>
+    </row>
+    <row r="8" ht="224" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>C006-P1</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr"/>
-      <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Oui on en a marre son équipe qui sûrement auront des comptes à rendre ...pour son parti politique violent..</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Encore melenchon purée quoi vous êtes pas fatigué 😅</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Acteur : autre
+Objet : violences et dégâts
+Position : condamne
+Preuve : pour son parti politique violent..
+Incertitude : ambigu
+Responsabilité attribuée : Parti et équipe de Mélenchon qualifiés de violents
+Argument : Mise en cause du parti dans le contexte du parent
+Note IA : La cible vient du parent et du titre. Pas de position explicite sur la police.</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="n"/>
+      <c r="I8" s="6" t="n"/>
+      <c r="J8" s="6" t="n"/>
+    </row>
+    <row r="9" ht="409" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>C007-P1</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr"/>
-      <c r="C9" s="2" t="inlineStr"/>
-      <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr"/>
-      <c r="G9" s="2" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Mr, depuis le 1 janvier 2009 grâce à Sarkozy, la République n'existe plus !
+Désolé, mais comprenez la vraie réalité.
+Depuis cette date, il n'y a plus que des fausses "lois Républicaines"..., une "fausse République" devenue "tyrannie" pour se maintenir au pouvoir... et rien d'autre !
+Et vous voulez respecter des"lois Républicaines" dans une "république" qui n'existe plus ?
+Ces manifestants, y compris les casseurs qui rentrent dans le jeu du "Macronistant", et dont je n'approuve en rien leurs comportements, n'ont pas conscience que nous sommes tous sous la contrainte et sous la propagande de 27 équipes de mafieux européennes, y compris les équipes de l'OTAN, de l'ONU, DAVOS, etc..., agissant en bande organisées contre les intérêts des peuples.
+Quand nous aurons tous compris, et réussi à expliquer la supercherie... On pourra mieux avancer...Tous ensemble ! 
+Force, vigilance, courage, respect à vous, et à tous pour retrouver ensemble notre vraie indépendance de notre Nation de France.</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>🤜🏻DIGNITÉ HONNEUR RESPECT🤛🏾
+COURAGES AUX POMPIERS QUI SONT LES VRAIS MILITAIRES PROTECTEURS DU PEUPLE ET DE TOUT LES PEUPLES.
+La responsabilité n´appartient ni de prêt ni de loin à LFI ... mais les medias trouvent une tête de turc... en ne cessant de parler de "l´extrême gauche" aux manettes...
+L´état est TOTALEMENT et DEFINITIVEMENT RESPONSABLE DE CE QU´IL SE PASSE !
+Faut arreter la mascarde !
+Trop de UAS UAS (Un Agent Smith) detiennent actuellement les commandes envers et contre toutes vraisemblances, des traitres à la nation, qui appartient celle ci, à tout ses citoyens, concitoyens, peuple, et population française en naissant libre et egaux (vous ne l´oterez pas et ni la fraternité au passage ...car ils cherchent et veulent fracturer le pays "diviser pour mieux régner") et de tout horizons aussi diverses que variés...!
+Ne pas se tromper d´ennemis et ni de combat...!
+Ceux qui en leurs âmes et consciences pensent, veulent et ou causent directement ou indirectement, du tort à la république et en entravant les lois républicaines, en paieront le prix et le lourd poids des conséquences en assumant leurs responsabilités, à un moment ou à un autre, l´histoire le conforte et le confirme (elle n´est qu´un eternelle recommencement...) ...
+Ce n´est qu´une simple question de temps.
+Il faut stopper toutes activités pro afin de paralyser toutes emoragies et on va voir ensuite ce qu´il se passe...!</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Acteur : manifestants
+Objet : violences et dégâts
+Position : condamne
+Preuve : dont je n'approuve en rien leurs comportements
+Incertitude : lecture explicite
+Argument : Désapprobation explicite de comportements attribués aux manifestants et casseurs
+Note IA : Ne pas importer dans cette réponse toutes les accusations formulées par le parent.</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="6" t="n"/>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="6" t="n"/>
+      <c r="I9" s="6" t="n"/>
+      <c r="J9" s="6" t="n"/>
+    </row>
+    <row r="10" ht="224" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>C008-P1</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr"/>
-      <c r="C10" s="2" t="inlineStr"/>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr"/>
-      <c r="G10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Bonjour, tu n’as rien compris… la police ne tabasse pas les retraités. Ils tabassent ceux qu’ils méritent d’être tabassés</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Bonjour, je suis Norvégien vivant en France et je ne comprend pas pourquoi chez vous la police tabasse constamment les mineurs, les retraités, les femmes, les étrangers mais jamais les casseurs... La seule explication rationnel que je trouve c'est que le gouvernement laisse les casseurs pour décrédibiliser complètement le mouvement et permettre à la police de charger encore plus les mineurs, les retraités, les femmes et les étrangers. Je pense que vos policiers et politiques ont des soucis psychologiques graves (j'ai vu une video d'un policier à Carcassonne, son âme était très moche)</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Acteur : police
+Objet : usage de la force
+Position : justifie ou soutient
+Preuve : Ils tabassent ceux qu’ils méritent d’être tabassés
+Incertitude : lecture explicite
+Argument : Les personnes frappées sont présentées comme méritant les coups
+Note IA : Rejet de l’accusation du parent; justification explicite, formulation conservée.</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
+      <c r="I10" s="6" t="n"/>
+      <c r="J10" s="6" t="n"/>
+    </row>
+    <row r="11" ht="196" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>C009-P1</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr"/>
-      <c r="C11" s="2" t="inlineStr"/>
-      <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Total soutien avec vous tous.tes. Tout le monde déteste la milice-police ! 
+Merci BG pour ce direct.</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Aucun parent : commentaire principal.</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Acteur : police
+Objet : autre
+Position : condamne
+Preuve : Tout le monde déteste la milice-police !
+Incertitude : lecture explicite
+Argument : Assimilation de la police à une milice
+Note IA : Hostilité générale exprimée; ne spécifie pas une intervention ni un usage de la force précis.</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="6" t="n"/>
+      <c r="H11" s="6" t="n"/>
+      <c r="I11" s="6" t="n"/>
+      <c r="J11" s="6" t="n"/>
+    </row>
+    <row r="12" ht="196" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>C009-P2</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr"/>
-      <c r="C12" s="2" t="inlineStr"/>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr"/>
-      <c r="G12" s="2" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Total soutien avec vous tous.tes. Tout le monde déteste la milice-police ! 
+Merci BG pour ce direct.</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Aucun parent : commentaire principal.</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Acteur : autre
+Objet : autre
+Position : justifie ou soutient
+Preuve : Total soutien avec vous tous.tes.
+Incertitude : contexte insuffisant
+Argument : Soutien collectif dans le contexte du direct
+Note IA : Le groupe soutenu n’est pas précisément identifié dans le texte; interprétation à vérifier.</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="n"/>
+      <c r="H12" s="6" t="n"/>
+      <c r="I12" s="6" t="n"/>
+      <c r="J12" s="6" t="n"/>
+    </row>
+    <row r="13" ht="196" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>C010-P1</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr"/>
-      <c r="C13" s="2" t="inlineStr"/>
-      <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr"/>
-      <c r="G13" s="2" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>C'est pour cela qu'il faut quoi qu'il en coûte ...protéger les pâtisseries de luxe du nord-ouest de la France avec moult CRS ! (Un minimum de 6 cars de ces défenseurs de la diabétique liberté est la préconisation)</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Aucun parent : commentaire principal.</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Acteur : police
+Objet : protection et sécurité
+Position : indéterminée
+Preuve : avec moult CRS !
+Incertitude : ambigu
+Argument : Protection de commerces de luxe évoquée sur un registre possiblement ironique
+Note IA : Ironie probable; ne pas convertir la demande littérale de protection en soutien certain à l’intervention.</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="6" t="n"/>
+      <c r="H13" s="6" t="n"/>
+      <c r="I13" s="6" t="n"/>
+      <c r="J13" s="6" t="n"/>
+    </row>
+    <row r="14" ht="196" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>C011-P1</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr"/>
-      <c r="C14" s="2" t="inlineStr"/>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr"/>
-      <c r="G14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>des faux policiers oui</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>J'espère qu'ils ont les vidéos des flics qui provoquent et cassent.</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Acteur : police
+Objet : violences et dégâts
+Position : nuance
+Preuve : des faux policiers oui
+Incertitude : ambigu
+Responsabilité attribuée : Actes du parent réattribués à de faux policiers
+Note IA : Le parent accuse des policiers de provoquer et casser; la réponse semble contester leur identité, sans preuve.</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="6" t="n"/>
+      <c r="H14" s="6" t="n"/>
+      <c r="I14" s="6" t="n"/>
+      <c r="J14" s="6" t="n"/>
+    </row>
+    <row r="15" ht="224" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>C012-P1</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr"/>
-      <c r="C15" s="2" t="inlineStr"/>
-      <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr"/>
-      <c r="G15" s="2" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>C’est fou les gens qui les défendent encore.   Ils ont tapé sur les gilets jaune.  Sur nos infirmiers, sur nos agriculteurs, sur les étudiants.   Mais certains pensent encore qu’ils font la part des choses entre manifestants et casseurs.</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Oui, tout à fait, merci aux forces de l'ordre pour la sécurité de nos jeunes dans la rue qui revendiquent légitimement. Non aux casseurs ! Et tous ceux qui les supportent et les mélangent sont responsables !</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Acteur : police
+Objet : usage de la force
+Position : condamne
+Preuve : Ils ont tapé sur les gilets jaune.
+Incertitude : lecture explicite
+Responsabilité attribuée : Forces de l’ordre accusées de frapper diverses catégories de manifestants
+Argument : Absence de distinction entre manifestants et casseurs
+Note IA : Le parent permet de résoudre le pronom « ils ». Ne pas attribuer à la réponse le soutien policier du parent.</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="6" t="n"/>
+      <c r="H15" s="6" t="n"/>
+      <c r="I15" s="6" t="n"/>
+      <c r="J15" s="6" t="n"/>
+    </row>
+    <row r="16" ht="224" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>C013-P1</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr"/>
-      <c r="C16" s="2" t="inlineStr"/>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr"/>
-      <c r="G16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>​@denischizallet818 C'est la vidéo qui parle précisément d'une rue, c'est pour ça que je précise une rue de Paris ou tout ce qui a été cassé samedi. Après si vous n'êtes pas capable de comprendre que l'immense majorité des manifestants a défilé dans le calme et que les pillages ne sont le fait que d'une minorité de casseurs, je peux rien pour vous.</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>C'est effectivement du grand n'importe quoi et il faut absolument être solidaire de tous les commerçants qui ont perdu leur outil de travail. Maintenant réduire toute la jeunesse du pays à une rue de Paris délabrée ou même à tout ce qui a été cassé hier, faut peut-être nuancer un peu. Les casseurs doivent être retrouvés et punis mais c'est pas en généralisant à toute une génération qu'on fera avancer ce pays...</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Acteur : manifestants
+Objet : violences et dégâts
+Position : nuance
+Preuve : l'immense majorité des manifestants a défilé dans le calme
+Incertitude : lecture explicite
+Responsabilité attribuée : Pillages attribués à une minorité de casseurs
+Argument : Distinction entre majorité pacifique et minorité violente
+Note IA : Nuance la généralisation de la violence à l’ensemble des manifestants.</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="6" t="n"/>
+      <c r="H16" s="6" t="n"/>
+      <c r="I16" s="6" t="n"/>
+      <c r="J16" s="6" t="n"/>
+    </row>
+    <row r="17" ht="196" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>C014-P1</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr"/>
-      <c r="C17" s="2" t="inlineStr"/>
-      <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="2" t="inlineStr"/>
-      <c r="F17" s="2" t="inlineStr"/>
-      <c r="G17" s="2" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>C’EST QUOI CES ROBOCOPS ? J’AI VU DES POLICIERS CAGOULÉS  ET CACHANT LEUR MATRICULE R. I.O AVEC DES INSIGNES NAZIS POUR CASSER ET PILLER ET PROVOQUER....!!!!!! Et AUCUNE TÉLÉ NE LE MONTRE...VOUS ÊTES TROP ORIENTÉS LES JOURNALISTES.... FASCISTE. LE SAVEZ-VOUS?</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Aucun parent : commentaire principal.</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Acteur : police
+Objet : violences et dégâts
+Position : condamne
+Preuve : POUR CASSER ET PILLER ET PROVOQUER
+Incertitude : lecture explicite
+Responsabilité attribuée : Policiers accusés de cacher leur identification et de participer aux dégradations
+Note IA : Accusations non vérifiées de l’auteur; aucune observation factuelle du rapport.</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n"/>
+      <c r="G17" s="6" t="n"/>
+      <c r="H17" s="6" t="n"/>
+      <c r="I17" s="6" t="n"/>
+      <c r="J17" s="6" t="n"/>
+    </row>
+    <row r="18" ht="224" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>C015-P1</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr"/>
-      <c r="C18" s="2" t="inlineStr"/>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr"/>
-      <c r="G18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>quand en face ils ont reçue de la violence(oeil crevé,mains arraché, machoir cassé) il faut pas s'attendre à ce que les gens restent pacifiques</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Aucun parent : commentaire principal.</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Acteur : autre
+Objet : violences et dégâts
+Position : justifie ou soutient
+Preuve : il faut pas s'attendre à ce que les gens restent pacifiques
+Incertitude : ambigu
+Responsabilité attribuée : Violences antérieures présentées comme cause d’une réaction non pacifique
+Argument : Blessures graves subies
+Note IA : Normalise une réaction violente possible; auteur des violences initiales non explicite, donc pas d’attribution certaine à la police.</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="n"/>
+      <c r="G18" s="6" t="n"/>
+      <c r="H18" s="6" t="n"/>
+      <c r="I18" s="6" t="n"/>
+      <c r="J18" s="6" t="n"/>
+    </row>
+    <row r="19" ht="224" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>C016-P1</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr"/>
-      <c r="C19" s="2" t="inlineStr"/>
-      <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="2" t="inlineStr"/>
-      <c r="F19" s="2" t="inlineStr"/>
-      <c r="G19" s="2" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Il faut parler de nos policiers qui font pipi sur les itinéraires, il faut régler nos problèmes et les laisser les problèmes des autre pays avant que sa pete même ici</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Aucun parent : commentaire principal.</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Acteur : police
+Objet : autre
+Position : condamne
+Preuve : nos policiers qui font pipi sur les itinéraires
+Incertitude : ambigu
+Responsabilité attribuée : Comportement inconvenant allégué de policiers
+Argument : Appel à régler des problèmes internes
+Note IA : Police mentionnée mais action décrite peu claire; pas de position certaine sur l’usage de la force.</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="n"/>
+      <c r="F19" s="6" t="n"/>
+      <c r="G19" s="6" t="n"/>
+      <c r="H19" s="6" t="n"/>
+      <c r="I19" s="6" t="n"/>
+      <c r="J19" s="6" t="n"/>
+    </row>
+    <row r="20" ht="196" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>C017-P1</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr"/>
-      <c r="C20" s="2" t="inlineStr"/>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr"/>
-      <c r="G20" s="2" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Mais vous avez complètement détourner le propos de Elise 😂 elle a surtout condamné la violence de la police</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Aucun parent : commentaire principal.</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Acteur : police
+Objet : usage de la force
+Position : indéterminée
+Preuve : elle a surtout condamné la violence de la police
+Incertitude : lecture explicite
+Argument : Rectification de la position d’une tierce personne
+Note IA : La condamnation est attribuée à Elise; l’adhésion de l’auteur n’est pas établie. Titre situant la vidéo à Marseille.</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="n"/>
+      <c r="G20" s="6" t="n"/>
+      <c r="H20" s="6" t="n"/>
+      <c r="I20" s="6" t="n"/>
+      <c r="J20" s="6" t="n"/>
+    </row>
+    <row r="21" ht="196" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>C018-P1</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr"/>
-      <c r="C21" s="2" t="inlineStr"/>
-      <c r="D21" s="2" t="inlineStr"/>
-      <c r="E21" s="2" t="inlineStr"/>
-      <c r="F21" s="2" t="inlineStr"/>
-      <c r="G21" s="2" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>La police devrait laisser tomber la france 48h tout laisser bruler</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Aucun parent : commentaire principal.</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Acteur : police
+Objet : protection et sécurité
+Position : indéterminée
+Preuve : La police devrait laisser tomber la france 48h tout laisser bruler
+Incertitude : ambigu
+Argument : Souhaite un retrait de la police avec perspective de destructions
+Note IA : Soutien littéral au retrait, pas nécessairement à l’abandon réel de la protection; hypothèse rhétorique à discuter. Exemple important pour revoir la grille.</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="n"/>
+      <c r="F21" s="6" t="n"/>
+      <c r="G21" s="6" t="n"/>
+      <c r="H21" s="6" t="n"/>
+      <c r="I21" s="6" t="n"/>
+      <c r="J21" s="6" t="n"/>
+    </row>
+    <row r="22" ht="196" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>C019-P1</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr"/>
-      <c r="C22" s="2" t="inlineStr"/>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr"/>
-      <c r="G22" s="2" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>C’est pas des tensions : c'est des violences urbaines et des pillages. Une agence de presse devrait appeler les choses par leur nom</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Aucun parent : commentaire principal.</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Acteur : autre
+Objet : violences et dégâts
+Position : condamne
+Preuve : c'est des violences urbaines et des pillages
+Incertitude : ambigu
+Argument : Rejet du terme atténué « tensions » pour décrire des pillages
+Note IA : Cible directe : cadrage médiatique; jugement sur les violences inféré avec prudence. Aucune position sur la police déduite.</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="n"/>
+      <c r="F22" s="6" t="n"/>
+      <c r="G22" s="6" t="n"/>
+      <c r="H22" s="6" t="n"/>
+      <c r="I22" s="6" t="n"/>
+      <c r="J22" s="6" t="n"/>
+    </row>
+    <row r="23" ht="196" customHeight="1">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>C020-P1</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr"/>
-      <c r="C23" s="2" t="inlineStr"/>
-      <c r="D23" s="2" t="inlineStr"/>
-      <c r="E23" s="2" t="inlineStr"/>
-      <c r="F23" s="2" t="inlineStr"/>
-      <c r="G23" s="2" t="inlineStr"/>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>OUI LFI ET SA MILICE ANTIFAS ORGANISENT LE PILLAGE</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Aucun parent : commentaire principal.</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Acteur : autre
+Objet : violences et dégâts
+Position : condamne
+Preuve : LFI ET SA MILICE ANTIFAS ORGANISENT LE PILLAGE
+Incertitude : lecture explicite
+Responsabilité attribuée : LFI et antifascistes accusés d’organiser les pillages
+Note IA : Attribution de responsabilité formulée par l’auteur, non vérifiée. Titre portant sur le 24 octobre; pertinence événementielle à vérifier.</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="n"/>
+      <c r="F23" s="6" t="n"/>
+      <c r="G23" s="6" t="n"/>
+      <c r="H23" s="6" t="n"/>
+      <c r="I23" s="6" t="n"/>
+      <c r="J23" s="6" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G23"/>
+  <autoFilter ref="A1:J23"/>
+  <dataValidations count="3">
+    <dataValidation sqref="E2:E23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"accord,désaccord,à discuter"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F2:F23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"police,manifestants,casseurs,gouvernement,autre,indéterminé"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"condamne,justifie ou soutient,nuance,décrit sans position,indéterminée"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>